<commit_message>
Update to perfect code count + other fixes
</commit_message>
<xml_diff>
--- a/tests/output_Rapport-Template-Soir.xlsx
+++ b/tests/output_Rapport-Template-Soir.xlsx
@@ -518,7 +518,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Exécuté le : 2026-08-30 03:08:40 | Quart : Soir</t>
+          <t>Exécuté le : 2026-08-31 02:15:48 | Quart : Soir</t>
         </is>
       </c>
       <c r="B2" s="1" t="n"/>
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -731,7 +731,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>Inf</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
@@ -755,20 +755,20 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>PAB</t>
+          <t>Aux</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="E6" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="F6" s="8" t="n">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -779,20 +779,20 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Inf</t>
+          <t>PAB</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -803,7 +803,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Aux</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="C8" s="7" t="n">
@@ -827,14 +827,14 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>PAB</t>
+          <t>Inf</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>0</v>
@@ -851,7 +851,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Inf</t>
+          <t>Aux</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
@@ -875,14 +875,14 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Aux</t>
+          <t>PAB</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E11" s="6" t="n">
         <v>0</v>
@@ -975,16 +975,16 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1019,20 +1019,20 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>PAB</t>
+          <t>Inf</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E17" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F17" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -1043,14 +1043,14 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>PAB</t>
+          <t>Aux</t>
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E18" s="7" t="n">
         <v>0</v>
@@ -1067,14 +1067,14 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Inf</t>
+          <t>PAB</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E19" s="6" t="n">
         <v>0</v>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Aux</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="C20" s="7" t="n">
@@ -1110,12 +1110,12 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>8e</t>
+          <t>SIC</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>Inf</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
@@ -1139,20 +1139,20 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>PAB</t>
+          <t>Aux</t>
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="E22" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="8" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -1163,20 +1163,20 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Inf</t>
+          <t>PAB</t>
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="6" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="E23" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Aux</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="C24" s="7" t="n">
@@ -1206,12 +1206,12 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>SIC</t>
+          <t>CDJ</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>Inf</t>
         </is>
       </c>
       <c r="C25" s="6" t="n">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Inf</t>
+          <t>Aux</t>
         </is>
       </c>
       <c r="C26" s="7" t="n">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Aux</t>
+          <t>PAB</t>
         </is>
       </c>
       <c r="C27" s="6" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>PAB</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="C28" s="7" t="n">
@@ -1302,12 +1302,12 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>CDJ</t>
+          <t>URG</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>Inf</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
@@ -1331,20 +1331,20 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>PAB</t>
+          <t>Aux</t>
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D30" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="8" t="n">
-        <v>-2</v>
-      </c>
-      <c r="F30" s="8" t="n">
-        <v>-2</v>
+        <v>0</v>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -1355,20 +1355,20 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Inf</t>
+          <t>PAB</t>
         </is>
       </c>
       <c r="C31" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="E31" s="8" t="n">
+        <v>-2</v>
+      </c>
+      <c r="F31" s="8" t="n">
+        <v>-2</v>
       </c>
     </row>
     <row r="32">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Aux</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="C32" s="7" t="n">
@@ -1398,12 +1398,12 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>URG</t>
+          <t>ECG</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>Inf</t>
         </is>
       </c>
       <c r="C33" s="6" t="n">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Inf</t>
+          <t>Aux</t>
         </is>
       </c>
       <c r="C34" s="7" t="n">
@@ -1451,7 +1451,7 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Aux</t>
+          <t>PAB</t>
         </is>
       </c>
       <c r="C35" s="6" t="n">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>PAB</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="C36" s="7" t="n">
@@ -1494,26 +1494,22 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>ECG</t>
+          <t>ACUR/GDL</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E37" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" s="6" t="n">
-        <v>0</v>
-      </c>
+          <t>Inf</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="D37" s="10" t="n"/>
+      <c r="E37" s="10" t="n"/>
+      <c r="F37" s="10" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -1523,7 +1519,7 @@
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>Aux</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
@@ -1543,7 +1539,7 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Inf</t>
+          <t>PAB</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
@@ -1563,7 +1559,7 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Aux</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">
@@ -1574,26 +1570,6 @@
       <c r="D40" s="10" t="n"/>
       <c r="E40" s="10" t="n"/>
       <c r="F40" s="10" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>ACUR/GDL</t>
-        </is>
-      </c>
-      <c r="B41" s="6" t="inlineStr">
-        <is>
-          <t>PAB</t>
-        </is>
-      </c>
-      <c r="C41" s="9" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="D41" s="10" t="n"/>
-      <c r="E41" s="10" t="n"/>
-      <c r="F41" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1602,14 +1578,14 @@
     <mergeCell ref="C39:F39"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="C38:F38"/>
-    <mergeCell ref="C41:F41"/>
+    <mergeCell ref="C37:F37"/>
   </mergeCells>
-  <conditionalFormatting sqref="E5:E41">
+  <conditionalFormatting sqref="E5:E40">
     <cfRule type="cellIs" priority="1" operator="notEqual" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F5:F41">
+  <conditionalFormatting sqref="F5:F40">
     <cfRule type="cellIs" priority="2" operator="notEqual" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -2468,7 +2444,7 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>Inf</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
@@ -2488,7 +2464,7 @@
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Inf</t>
+          <t>Aux</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
@@ -2508,7 +2484,7 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Aux</t>
+          <t>PAB</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
@@ -2528,7 +2504,7 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>PAB</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">

</xml_diff>

<commit_message>
fix(parser): align output with Sept 4th Gold Standard XLSX
</commit_message>
<xml_diff>
--- a/tests/output_Rapport-Template-Soir.xlsx
+++ b/tests/output_Rapport-Template-Soir.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet name="Rapport_Audit" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Le vendredi 4 sept. 2026" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="4 sept. 2026" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -91,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -114,6 +113,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -512,7 +514,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Exécuté le : 2026-09-01 01:00:01 | Quart : Soir</t>
+          <t>Exécuté le : 2026-09-01 22:50:29 | Quart : Soir</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -561,39 +563,31 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>21</v>
+        <v>64</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>23</v>
+        <v>63</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>4 sept. 2026</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>-5</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n"/>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Journal des anomalies</t>
+        </is>
+      </c>
       <c r="B7" s="3" t="n"/>
       <c r="C7" s="3" t="n"/>
       <c r="D7" s="3" t="n"/>
@@ -602,7 +596,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Journal des anomalies</t>
+          <t>Valeur Cible OCR improbable [Le vendredi 4 sept. 2026 | Soir | 4e | Aux] : 22 remplacée par 0.</t>
         </is>
       </c>
       <c r="B8" s="3" t="n"/>
@@ -613,7 +607,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Valeur Cible OCR improbable [Le vendredi 4 sept. 2026 | Soir | ACUR/GDL | AA] : 5315 remplacée par 0.</t>
+          <t>Écart détecté [Le vendredi 4 sept. 2026 | Soir | CDJ | Aux] : Présences indiquées = 4, Lignes comptées = 1. La valeur 1 a été retenue pour le fichier Excel.</t>
         </is>
       </c>
       <c r="B9" s="3" t="n"/>
@@ -622,10 +616,11 @@
       <c r="E9" s="3" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A8:E8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -709,10 +704,10 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E5" s="7" t="n">
         <v>0</v>
@@ -730,10 +725,10 @@
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>0</v>
@@ -754,10 +749,10 @@
         <v>2</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="E7" s="9" t="n">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -775,10 +770,10 @@
         <v>1</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="E8" s="9" t="n">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -793,10 +788,10 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>0</v>
@@ -814,10 +809,10 @@
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E10" s="8" t="n">
         <v>0</v>
@@ -859,10 +854,10 @@
         <v>1</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="9" t="n">
-        <v>-1</v>
+        <v>1</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -877,10 +872,10 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E13" s="7" t="n">
         <v>0</v>
@@ -898,10 +893,10 @@
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E14" s="8" t="n">
         <v>0</v>
@@ -943,10 +938,10 @@
         <v>1</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="9" t="n">
-        <v>-1</v>
+        <v>1</v>
+      </c>
+      <c r="E16" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -961,10 +956,10 @@
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E17" s="7" t="n">
         <v>0</v>
@@ -982,10 +977,10 @@
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E18" s="8" t="n">
         <v>0</v>
@@ -1027,10 +1022,10 @@
         <v>1</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="9" t="n">
-        <v>-1</v>
+        <v>1</v>
+      </c>
+      <c r="E20" s="8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -1045,10 +1040,10 @@
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D21" s="7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E21" s="7" t="n">
         <v>0</v>
@@ -1087,10 +1082,10 @@
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E23" s="7" t="n">
         <v>0</v>
@@ -1129,10 +1124,10 @@
         </is>
       </c>
       <c r="C25" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E25" s="7" t="n">
         <v>0</v>
@@ -1150,10 +1145,10 @@
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E26" s="8" t="n">
         <v>0</v>
@@ -1213,13 +1208,15 @@
         </is>
       </c>
       <c r="C29" s="7" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="D29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" s="7" t="n">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>0+HOR12</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -1234,10 +1231,10 @@
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E30" s="8" t="n">
         <v>0</v>
@@ -1255,13 +1252,13 @@
         </is>
       </c>
       <c r="C31" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D31" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E31" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -1339,10 +1336,10 @@
         </is>
       </c>
       <c r="C35" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D35" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E35" s="7" t="n">
         <v>0</v>
@@ -1451,842 +1448,6 @@
       </c>
       <c r="E40" s="8" t="n">
         <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
-  <conditionalFormatting sqref="E5:E40">
-    <cfRule type="cellIs" priority="1" operator="notEqual" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E40"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Soir</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="n"/>
-      <c r="C1" s="4" t="n"/>
-      <c r="D1" s="4" t="n"/>
-      <c r="E1" s="4" t="n"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>4 sept. 2026</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="n"/>
-      <c r="C2" s="5" t="n"/>
-      <c r="D2" s="5" t="n"/>
-      <c r="E2" s="5" t="n"/>
-    </row>
-    <row r="3"/>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Département</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Catégorie</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Cible</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Présences</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>Écart (Décompte vs Cible)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>4e</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>4e</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Aux</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>4e</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>PAB</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>4e</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="9" t="n">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>7e</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>7e</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Aux</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>7e</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>PAB</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>7e</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="9" t="n">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>6e</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>6e</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Aux</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>6e</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>PAB</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>6e</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="9" t="n">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>8e</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>8e</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Aux</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>8e</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>PAB</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>8e</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="9" t="n">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>SIC</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>SIC</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>Aux</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>SIC</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>PAB</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>SIC</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>CDJ</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>CDJ</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="inlineStr">
-        <is>
-          <t>Aux</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>CDJ</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>PAB</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>CDJ</t>
-        </is>
-      </c>
-      <c r="B28" s="8" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>URG</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>URG</t>
-        </is>
-      </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>Aux</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" s="8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>URG</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>PAB</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t>URG</t>
-        </is>
-      </c>
-      <c r="B32" s="8" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="C32" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D32" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" s="9" t="n">
-        <v>-2</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>ECG</t>
-        </is>
-      </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D33" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
-        <is>
-          <t>ECG</t>
-        </is>
-      </c>
-      <c r="B34" s="8" t="inlineStr">
-        <is>
-          <t>Aux</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D34" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" s="8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>ECG</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>PAB</t>
-        </is>
-      </c>
-      <c r="C35" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D35" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>ECG</t>
-        </is>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E36" s="8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="7" t="inlineStr">
-        <is>
-          <t>ACUR/GDL</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E37" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>ACUR/GDL</t>
-        </is>
-      </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>Aux</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E38" s="8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="7" t="inlineStr">
-        <is>
-          <t>ACUR/GDL</t>
-        </is>
-      </c>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>PAB</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E39" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
-        <is>
-          <t>ACUR/GDL</t>
-        </is>
-      </c>
-      <c r="B40" s="8" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D40" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E40" s="9" t="n">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(parser): handle page/date transitions, merge ACUR/GDL blocks, fix 6e anchor and apply HOR12/TRANS deduction rules
</commit_message>
<xml_diff>
--- a/tests/output_Rapport-Template-Soir.xlsx
+++ b/tests/output_Rapport-Template-Soir.xlsx
@@ -81,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -101,9 +101,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -502,7 +499,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Exécuté le : 2026-09-02 19:57:17 | Quart : Soir</t>
+          <t>Exécuté le : 2026-09-03 01:08:01 | Quart : Soir</t>
         </is>
       </c>
       <c r="B2" s="1" t="n"/>
@@ -551,13 +548,13 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
@@ -1177,10 +1174,8 @@
       <c r="D29" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="E29" s="9" t="inlineStr">
-        <is>
-          <t>1+HOR12</t>
-        </is>
+      <c r="E29" s="8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -1405,13 +1400,13 @@
         </is>
       </c>
       <c r="C40" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D40" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E40" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>